<commit_message>
Refine RAG control plane and evaluation
</commit_message>
<xml_diff>
--- a/docs/planning/to-adopt/Factored_decisiones.xlsx
+++ b/docs/planning/to-adopt/Factored_decisiones.xlsx
@@ -817,7 +817,7 @@
       </c>
       <c r="C13" s="11" t="inlineStr">
         <is>
-          <t>Implementar el workflow online determinista con LangGraph.js en el backend Bun/TypeScript, sin subagentes autónomos.</t>
+          <t>Implementar el workflow online determinista con LangGraph.js StateGraph en el backend Bun/TypeScript.</t>
         </is>
       </c>
       <c r="D13" s="10" t="inlineStr">
@@ -827,7 +827,7 @@
       </c>
       <c r="E13" s="11" t="inlineStr">
         <is>
-          <t>Fuente: directiva vigente. Fastify/Zod y @langchain/langgraph controlan estados, gates y políticas; DeepAgents queda limitado a evaluación offline.</t>
+          <t>StateGraph reúne nodos tipados y aristas condicionales; no hay subagentes autónomos. #TODO decidir más adelante ReAct preconstruido o loop propio, siempre mediado por policy.</t>
         </is>
       </c>
     </row>
@@ -842,7 +842,7 @@
       </c>
       <c r="C14" s="11" t="inlineStr">
         <is>
-          <t>Usar JEV para clasificar intención, riesgo y ruta; el Policy Engine decide aclaración, denegación, escalamiento o continuación.</t>
+          <t>Usar un JEV primario para clasificar llm, database, relations u ood; usar JEV especializado para cada RAG.</t>
         </is>
       </c>
       <c r="D14" s="10" t="inlineStr">
@@ -852,7 +852,7 @@
       </c>
       <c r="E14" s="11" t="inlineStr">
         <is>
-          <t>Fuente: Structured-RAG.md, KG RAG.md y referencia-agent-escalable-gcp.md. Incluye manejo de off-domain, baja comprensión y prompt injection antes de cualquier acción sensible.</t>
+          <t>Ambigüedad y baja confianza pasan a policy/aclaración. database conduce a Structured RAG; relations a KG-RAG. JEV no autoriza ni ejecuta.</t>
         </is>
       </c>
     </row>
@@ -942,7 +942,7 @@
       </c>
       <c r="C18" s="11" t="inlineStr">
         <is>
-          <t>Usar Structured RAG en TypeScript/Bun mediante @google-cloud/bigquery y un catálogo cerrado de templates BigQuery SELECT parametrizados y autorizados.</t>
+          <t>Usar Structured RAG en TypeScript/Bun mediante catálogo cerrado de QueryPlan BigQuery.</t>
         </is>
       </c>
       <c r="D18" s="10" t="inlineStr">
@@ -952,7 +952,7 @@
       </c>
       <c r="E18" s="11" t="inlineStr">
         <is>
-          <t>Fuente: Structured-RAG.md y directiva vigente. El backend Zod valida query_id, parámetros, tenant, costo y EvidenceDTO; no hay SQL libre.</t>
+          <t>El catálogo versionado se carga antes del JEV especializado; Zod valida query_id, parámetros, tenant y EvidenceDTO. No hay SQL libre ni vector-RAG.</t>
         </is>
       </c>
     </row>
@@ -967,7 +967,7 @@
       </c>
       <c r="C19" s="11" t="inlineStr">
         <is>
-          <t>Usar KG-RAG en TypeScript/Bun mediante un catálogo versionado de operaciones y artefactos de grafo compilados por el pipeline Python.</t>
+          <t>Usar KG-RAG en TypeScript/Bun mediante catálogo versionado de operaciones y artefactos de grafo compilados offline.</t>
         </is>
       </c>
       <c r="D19" s="10" t="inlineStr">
@@ -977,7 +977,7 @@
       </c>
       <c r="E19" s="11" t="inlineStr">
         <is>
-          <t>Fuente: KG RAG.md y directiva vigente. El backend valida operation_id con Zod, carga graph-vN.msgpack desde GCS y nunca acepta consultas de grafo libres.</t>
+          <t>KG-RAG carga obligatoriamente su catálogo de opciones antes de invocar su JEV especializado. Repository/adaptador queda #TODO y falla cerrado hasta conectar GCS, manifest y graph-vN.msgpack.</t>
         </is>
       </c>
     </row>
@@ -1202,7 +1202,7 @@
       </c>
       <c r="E28" s="11" t="inlineStr">
         <is>
-          <t>Fuente: referencia-agent-escalable-gcp.md. Mantiene frontend, autenticación y despliegue en la misma plataforma y reduce integraciones externas.</t>
+          <t>Firebase App Hosting es el único hosting frontend aprobado; Vercel queda fuera de alcance.</t>
         </is>
       </c>
     </row>
@@ -1317,7 +1317,7 @@
       </c>
       <c r="C33" s="11" t="inlineStr">
         <is>
-          <t>Guardar observabilidad y evaluación saneadas desde TypeScript/Bun en BigQuery; usar OpenTelemetry, DeepAgents y JEV-as-Judge solo en evaluación.</t>
+          <t>Usar evaluadores TypeScript propios, JEV-as-judge, OpenTelemetry y BigQuery para evaluación y observabilidad saneadas.</t>
         </is>
       </c>
       <c r="D33" s="10" t="inlineStr">
@@ -1327,7 +1327,7 @@
       </c>
       <c r="E33" s="11" t="inlineStr">
         <is>
-          <t>Fuente: referencia-agent-escalable-gcp.md y directiva vigente. Logs estructurados no incluyen prompts crudos, PII, audio, cookies, handles ni secretos.</t>
+          <t>docs/planning/evals.md prevalece: no incorporar LangSmith, DeepEval, Promptfoo ni DeepAgents en P0. Evaluadores de Structured RAG y KG-RAG extienden una base con invariantes de catálogo/evidencia.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Document invocation guides and refine agent evaluation
</commit_message>
<xml_diff>
--- a/docs/planning/to-adopt/Factored_decisiones.xlsx
+++ b/docs/planning/to-adopt/Factored_decisiones.xlsx
@@ -493,7 +493,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:E37"/>
+  <dimension ref="A1:E41"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="7" customWidth="1" style="5" min="1" max="1"/>
@@ -1317,7 +1317,7 @@
       </c>
       <c r="C33" s="11" t="inlineStr">
         <is>
-          <t>Usar evaluadores TypeScript propios, JEV-as-judge, OpenTelemetry y BigQuery para evaluación y observabilidad saneadas.</t>
+          <t>Usar evaluadores TypeScript propios, JEV-as-judge primero, LLM-as-judge opcional, OpenTelemetry y BigQuery para evaluación saneada.</t>
         </is>
       </c>
       <c r="D33" s="10" t="inlineStr">
@@ -1327,7 +1327,7 @@
       </c>
       <c r="E33" s="11" t="inlineStr">
         <is>
-          <t>docs/planning/evals.md prevalece: no incorporar LangSmith, DeepEval, Promptfoo ni DeepAgents en P0. Evaluadores de Structured RAG y KG-RAG extienden una base con invariantes de catálogo/evidencia.</t>
+          <t>ADR 0015 define EvaluationContext/EvaluationResult: score 0..1, passed, label, reasonCode allowlisted, evaluator/version/mode. P0 reporta scores informativos, ejecuta base una vez más override por ruta y no usa Docker adicional, LangSmith, DeepEval, Promptfoo, AgentEvals ni DeepAgents. Promptfoo queda como job CI efímero futuro, con versión fijada, si se requiere una batería end-to-end amplia o red-team.</t>
         </is>
       </c>
     </row>
@@ -1431,10 +1431,106 @@
         </is>
       </c>
     </row>
-    <row r="38" ht="27.75" customHeight="1" s="6"/>
-    <row r="39" ht="27.75" customHeight="1" s="6"/>
-    <row r="40" ht="15" customHeight="1" s="6"/>
-    <row r="41" ht="27.75" customHeight="1" s="6"/>
+    <row r="38" ht="27.75" customHeight="1" s="6">
+      <c r="A38" s="10" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" s="11" t="inlineStr">
+        <is>
+          <t>Evaluación / Release</t>
+        </is>
+      </c>
+      <c r="C38" s="11" t="inlineStr">
+        <is>
+          <t>Evaluar el agente por trayectoria, componente y end-to-end con golden set sintético versionado.</t>
+        </is>
+      </c>
+      <c r="D38" s="10" t="inlineStr">
+        <is>
+          <t>Definido</t>
+        </is>
+      </c>
+      <c r="E38" s="11" t="inlineStr">
+        <is>
+          <t>La matriz P0 tiene 48 fixtures: 12 rutas, 8 aclaración/policy/HITL, 10 Structured RAG, 10 KG-RAG y 8 seguridad/resiliencia. Gates de calidad son informativos hasta una línea base revisada por humano.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="27.75" customHeight="1" s="6">
+      <c r="A39" s="10" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" s="11" t="inlineStr">
+        <is>
+          <t>Datos / Pipeline</t>
+        </is>
+      </c>
+      <c r="C39" s="11" t="inlineStr">
+        <is>
+          <t>Usar un pipeline offline Python 3.12 en Cloud Run Job para transferir S3 a GCS, cargar BigQuery, ejecutar KDD/Naive Bayes y publicar el grafo.</t>
+        </is>
+      </c>
+      <c r="D39" s="10" t="inlineStr">
+        <is>
+          <t>Definido</t>
+        </is>
+      </c>
+      <c r="E39" s="11" t="inlineStr">
+        <is>
+          <t>ADR 0020. Storage Transfer Service mueve S3→GCS sin agentes; cada run-id conserva manifest, checksum, lineage y calidad. KDD/Naive Bayes son señales exploratorias, nunca autorización online. Solo una publicación validada actualiza graph-vN.msgpack y current.json.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="15" customHeight="1" s="6">
+      <c r="A40" s="10" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" s="11" t="inlineStr">
+        <is>
+          <t>Frontend / Despliegue</t>
+        </is>
+      </c>
+      <c r="C40" s="11" t="inlineStr">
+        <is>
+          <t>Usar Next.js 15.2, React, TypeScript y Tailwind para cliente/backoffice, entregado exclusivamente por Firebase App Hosting.</t>
+        </is>
+      </c>
+      <c r="D40" s="10" t="inlineStr">
+        <is>
+          <t>Definido</t>
+        </is>
+      </c>
+      <c r="E40" s="11" t="inlineStr">
+        <is>
+          <t>ADR 0021. Firebase Auth entrega identidad y Cloud Run conserva autorización. Vercel queda fuera de alcance; frontend no consulta almacenes de datos directamente ni expone secretos en NEXT_PUBLIC_*.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="27.75" customHeight="1" s="6">
+      <c r="A41" s="10" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" s="11" t="inlineStr">
+        <is>
+          <t>Datos / Trazabilidad incremental</t>
+        </is>
+      </c>
+      <c r="C41" s="11" t="inlineStr">
+        <is>
+          <t>Cerrar la ingesta con reconciliación S3→GCS, Eventarc, Cloud Tasks idempotentes, ledger BigQuery y refresh serializado del pipeline.</t>
+        </is>
+      </c>
+      <c r="D41" s="10" t="inlineStr">
+        <is>
+          <t>Definido</t>
+        </is>
+      </c>
+      <c r="E41" s="11" t="inlineStr">
+        <is>
+          <t>ADR 0020, ADR 0014 y ADR 0017. Scheduler reconcilia cada 15 min con lookback 30 min; Eventarc dispara dispatcher al finalizar GCS; Cloud Task verifica y carga raw/ledger. Firestore serializa KDD/publicación y ningún fallo actualiza current.json.</t>
+        </is>
+      </c>
+    </row>
     <row r="42" ht="27.75" customHeight="1" s="6"/>
     <row r="43" ht="27.75" customHeight="1" s="6"/>
     <row r="44" ht="27.75" customHeight="1" s="6"/>

</xml_diff>

<commit_message>
chore: consolidate KG pipeline and task clarity
</commit_message>
<xml_diff>
--- a/docs/planning/to-adopt/Factored_decisiones.xlsx
+++ b/docs/planning/to-adopt/Factored_decisiones.xlsx
@@ -842,7 +842,7 @@
       </c>
       <c r="C14" s="11" t="inlineStr">
         <is>
-          <t>Usar un JEV primario para clasificar llm, database, relations u ood; usar JEV especializado para cada RAG.</t>
+          <t>Usar un JEV primario para clasificar llm, database, relations u ood; usar JEV especializado para cada RAG sobre una proyección tipada mínima.</t>
         </is>
       </c>
       <c r="D14" s="10" t="inlineStr">
@@ -852,7 +852,7 @@
       </c>
       <c r="E14" s="11" t="inlineStr">
         <is>
-          <t>Ambigüedad y baja confianza pasan a policy/aclaración. database conduce a Structured RAG; relations a KG-RAG. JEV no autoriza ni ejecuta.</t>
+          <t>Ambigüedad y baja confianza pasan a policy/aclaración. Las instrucciones, opciones, identidad y catálogo son controlados por backend; texto de usuario, memoria y recuperación son estado no confiable y no autorizan ni ejecutan.</t>
         </is>
       </c>
     </row>
@@ -1067,7 +1067,7 @@
       </c>
       <c r="C23" s="11" t="inlineStr">
         <is>
-          <t>Aplicar Model Armor a entrada y salida con plantillas separadas; calibrar primero en modo Inspect only y bloquear después según policy.</t>
+          <t>Aplicar Model Armor a entrada y salida con plantillas separadas, y proteger la proyección JEV de contenido indirecto no confiable.</t>
         </is>
       </c>
       <c r="D23" s="10" t="inlineStr">
@@ -1077,7 +1077,7 @@
       </c>
       <c r="E23" s="11" t="inlineStr">
         <is>
-          <t>Fuente: documentación oficial de Model Armor. Protege contra prompt injection, jailbreak, URLs maliciosas y exposición de PII; los eventos alimentan el ajuste de umbrales.</t>
+          <t>Calibrar primero en modo Inspect only y bloquear después según policy. Opiniones, instrucciones, autoridad, recuperación y campos fuera de schema no pueden ampliar rutas, permisos ni catálogo.</t>
         </is>
       </c>
     </row>
@@ -1092,7 +1092,7 @@
       </c>
       <c r="C24" s="11" t="inlineStr">
         <is>
-          <t>Persistir únicamente contenido, evidencia y telemetría previamente saneados.</t>
+          <t>Persistir únicamente evidencia y telemetría previamente saneadas; exportar trazas sólo como metadata allowlisted.</t>
         </is>
       </c>
       <c r="D24" s="10" t="inlineStr">
@@ -1102,7 +1102,7 @@
       </c>
       <c r="E24" s="11" t="inlineStr">
         <is>
-          <t>Fuente: referencia-agent-escalable-gcp.md. No se almacenan prompts crudos, secretos, handles, PII no autorizada ni datos de sesión como trazabilidad durable.</t>
+          <t>No se almacenan prompts crudos, secretos, handles, PII no autorizada ni datos de sesión. Tenant, sesión, usuario y correlación externa se pseudonimizan con HMAC rotado.</t>
         </is>
       </c>
     </row>
@@ -1317,7 +1317,7 @@
       </c>
       <c r="C33" s="11" t="inlineStr">
         <is>
-          <t>Usar evaluadores TypeScript propios, JEV-as-judge primero, LLM-as-judge opcional, OpenTelemetry y BigQuery para evaluación saneada.</t>
+          <t>Usar evaluadores TypeScript propios, JEV-as-judge primero, LLM-as-judge opcional, OpenTelemetry y Langfuse Cloud US para evaluación y trazabilidad saneadas.</t>
         </is>
       </c>
       <c r="D33" s="10" t="inlineStr">
@@ -1327,7 +1327,7 @@
       </c>
       <c r="E33" s="11" t="inlineStr">
         <is>
-          <t>ADR 0015 define EvaluationContext/EvaluationResult: score 0..1, passed, label, reasonCode allowlisted, evaluator/version/mode. P0 reporta scores informativos, ejecuta base una vez más override por ruta y no usa Docker adicional, LangSmith, DeepEval, Promptfoo, AgentEvals ni DeepAgents. Promptfoo queda como job CI efímero futuro, con versión fijada, si se requiere una batería end-to-end amplia o red-team.</t>
+          <t>ADR 0015 conserva EvaluationContext/EvaluationResult y el runner TypeScript como fuente de scores. Langfuse visualiza sólo spans y métricas allowlisted mediante OTel; no recibe contenido, no autoriza y no sustituye BigQuery. No se usa Docker, LangSmith, DeepEval, Promptfoo, AgentEvals ni DeepAgents en P0.</t>
         </is>
       </c>
     </row>
@@ -1342,7 +1342,7 @@
       </c>
       <c r="C34" s="11" t="inlineStr">
         <is>
-          <t>Optimizar costo con Firebase App Hosting, Cloud Run para backend Bun y Cloud Run Jobs Python, servicios administrados y scale-to-zero.</t>
+          <t>Optimizar costo con Firebase App Hosting, Cloud Run para backend Bun y Cloud Run Jobs Python, servicios administrados, scale-to-zero y observabilidad Cloud sin Docker adicional.</t>
         </is>
       </c>
       <c r="D34" s="10" t="inlineStr">
@@ -1352,7 +1352,7 @@
       </c>
       <c r="E34" s="11" t="inlineStr">
         <is>
-          <t>Fuente: directiva vigente. La transferencia S3→GCS es administrada; no se despliegan servicios Python online ni Kubernetes.</t>
+          <t>Langfuse Cloud US Hobby se activa sólo tras revisar región, retención, DPA, presupuesto de unidades y secretos en Secret Manager; no se autoalojará Langfuse durante la hackathon.</t>
         </is>
       </c>
     </row>
@@ -1442,7 +1442,7 @@
       </c>
       <c r="C38" s="11" t="inlineStr">
         <is>
-          <t>Evaluar el agente por trayectoria, componente y end-to-end con golden set sintético versionado.</t>
+          <t>Evaluar el agente por trayectoria, componente y end-to-end con golden set sintético versionado, CI determinista y regresión JEV opt-in.</t>
         </is>
       </c>
       <c r="D38" s="10" t="inlineStr">
@@ -1452,7 +1452,7 @@
       </c>
       <c r="E38" s="11" t="inlineStr">
         <is>
-          <t>La matriz P0 tiene 48 fixtures: 12 rutas, 8 aclaración/policy/HITL, 10 Structured RAG, 10 KG-RAG y 8 seguridad/resiliencia. Gates de calidad son informativos hasta una línea base revisada por humano.</t>
+          <t>La matriz P0 conserva 48 fixtures core y las extensiones KG. PR bloquea contratos y pruebas deterministas; JEV real sólo corre manual/nocturno sobre fixtures sintéticos y reporta ruido de rerun, flips, drift y confianza hasta contar con baseline humana.</t>
         </is>
       </c>
     </row>

</xml_diff>